<commit_message>
Add profiling fine tunings
</commit_message>
<xml_diff>
--- a/evaluations/response_time_increasing_clients/1_DB/aggregated_workload.xlsx
+++ b/evaluations/response_time_increasing_clients/1_DB/aggregated_workload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\evaluations\response_time_increasing_clients\1_DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCB6F3E-93CD-4BA6-8830-B1CFF24B0B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C6492B-9F3D-414A-AF73-D956E02621E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>User Count</t>
   </si>
@@ -46,12 +46,15 @@
   <si>
     <t>Growth Rate Response Time</t>
   </si>
+  <si>
+    <t>Linear Growth Rate</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,6 +66,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -72,16 +76,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -113,22 +130,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -428,15 +463,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -449,8 +486,11 @@
       <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -464,8 +504,12 @@
         <f>C3/C2</f>
         <v>1.4406098115354042</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <f>C3-C2</f>
+        <v>4.4831763662749999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -476,11 +520,15 @@
         <v>14.658111760138249</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E51" si="0">C4/C3</f>
+        <f t="shared" ref="E3:E50" si="0">C4/C3</f>
         <v>1.4058226864590255</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f t="shared" ref="F3:F49" si="1">C4-C3</f>
+        <v>5.9485942929159403</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -494,8 +542,12 @@
         <f t="shared" si="0"/>
         <v>1.3260926096351164</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>6.7196945528241905</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -509,8 +561,12 @@
         <f t="shared" si="0"/>
         <v>1.2142772760459457</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>5.8554266859679025</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -524,8 +580,12 @@
         <f t="shared" si="0"/>
         <v>1.2100790364016394</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>6.9708063035166887</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -539,8 +599,12 @@
         <f t="shared" si="0"/>
         <v>1.1707148366735165</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>6.8546502862439453</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -554,8 +618,12 @@
         <f t="shared" si="0"/>
         <v>1.139596547025908</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>6.5620545149389429</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -569,8 +637,12 @@
         <f t="shared" si="0"/>
         <v>1.1321886438302369</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <f t="shared" si="1"/>
+        <v>7.0812581935224372</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -584,8 +656,12 @@
         <f t="shared" si="0"/>
         <v>1.1030461211825802</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>6.2498087260159636</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -599,8 +675,12 @@
         <f t="shared" si="0"/>
         <v>1.1031536413610059</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>6.9010204168812948</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -614,8 +694,12 @@
         <f t="shared" si="0"/>
         <v>1.0859315015340771</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>6.3418673285894158</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -629,8 +713,12 @@
         <f t="shared" si="0"/>
         <v>1.0813070893991934</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>6.516217893701608</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -644,8 +732,12 @@
         <f t="shared" si="0"/>
         <v>1.0825782268733364</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>7.1561887563955651</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -659,8 +751,12 @@
         <f t="shared" si="0"/>
         <v>1.0741215651334899</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>6.9537664967211583</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -674,8 +770,12 @@
         <f t="shared" si="0"/>
         <v>1.0665304960086324</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16">
+        <f t="shared" si="1"/>
+        <v>6.7042425693682048</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -689,8 +789,12 @@
         <f t="shared" si="0"/>
         <v>1.0623402760950154</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17">
+        <f t="shared" si="1"/>
+        <v>6.6999406781596917</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -704,8 +808,12 @@
         <f t="shared" si="0"/>
         <v>1.0549244527735484</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <f t="shared" si="1"/>
+        <v>6.270925217524308</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -719,8 +827,12 @@
         <f t="shared" si="0"/>
         <v>1.0488149624533203</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <f t="shared" si="1"/>
+        <v>5.879497390389389</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -734,8 +846,12 @@
         <f t="shared" si="0"/>
         <v>1.0470229881212256</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <f t="shared" si="1"/>
+        <v>5.9401353400816106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -749,8 +865,12 @@
         <f t="shared" si="0"/>
         <v>1.0448773121735484</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21">
+        <f t="shared" si="1"/>
+        <v>5.9356621250516071</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -764,8 +884,12 @@
         <f t="shared" si="0"/>
         <v>1.0447174437619762</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22">
+        <f t="shared" si="1"/>
+        <v>6.1799448935731789</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -779,8 +903,12 @@
         <f t="shared" si="0"/>
         <v>1.0485828034243259</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <f t="shared" si="1"/>
+        <v>7.0143761425300113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -794,8 +922,12 @@
         <f t="shared" si="0"/>
         <v>1.0433125956700477</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24">
+        <f t="shared" si="1"/>
+        <v>6.5572753627382099</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -809,8 +941,12 @@
         <f t="shared" si="0"/>
         <v>1.0479593643450347</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25">
+        <f t="shared" si="1"/>
+        <v>7.5752519032631938</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -824,8 +960,12 @@
         <f t="shared" si="0"/>
         <v>1.0395378243792817</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26">
+        <f t="shared" si="1"/>
+        <v>6.5445662996830833</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -839,8 +979,12 @@
         <f t="shared" si="0"/>
         <v>1.0344218278085571</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <f t="shared" si="1"/>
+        <v>5.9230081131454995</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -854,8 +998,12 @@
         <f t="shared" si="0"/>
         <v>1.0373437476459098</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28">
+        <f t="shared" si="1"/>
+        <v>6.6469739319678069</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -869,8 +1017,12 @@
         <f t="shared" si="0"/>
         <v>1.0334797155633249</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29">
+        <f t="shared" si="1"/>
+        <v>6.1817370728196011</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -884,8 +1036,12 @@
         <f t="shared" si="0"/>
         <v>1.0351080477805281</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30">
+        <f t="shared" si="1"/>
+        <v>6.6994231156781154</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -899,8 +1055,12 @@
         <f t="shared" si="0"/>
         <v>1.0353748271352701</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31">
+        <f t="shared" si="1"/>
+        <v>6.9873216879778965</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -914,8 +1074,12 @@
         <f t="shared" si="0"/>
         <v>1.0332287586322169</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32">
+        <f t="shared" si="1"/>
+        <v>6.7956050559661776</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -929,8 +1093,12 @@
         <f t="shared" si="0"/>
         <v>1.026743825872215</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33">
+        <f t="shared" si="1"/>
+        <v>5.6511135693950223</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -944,8 +1112,12 @@
         <f t="shared" si="0"/>
         <v>1.031476695982648</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34">
+        <f t="shared" si="1"/>
+        <v>6.8290727430830032</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -959,8 +1131,12 @@
         <f t="shared" si="0"/>
         <v>1.0286122438191028</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35">
+        <f t="shared" si="1"/>
+        <v>6.403006417096492</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -974,8 +1150,12 @@
         <f t="shared" si="0"/>
         <v>1.0316862535749451</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36">
+        <f t="shared" si="1"/>
+        <v>7.2938126334665014</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -989,8 +1169,12 @@
         <f t="shared" si="0"/>
         <v>1.0292856291238246</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37">
+        <f t="shared" si="1"/>
+        <v>6.9548202736425822</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1004,8 +1188,12 @@
         <f t="shared" si="0"/>
         <v>1.0288706836836972</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <f t="shared" si="1"/>
+        <v>7.0570684680815248</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1019,8 +1207,12 @@
         <f t="shared" si="0"/>
         <v>1.0275313260393875</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39">
+        <f t="shared" si="1"/>
+        <v>6.9239701170529599</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1034,8 +1226,12 @@
         <f t="shared" si="0"/>
         <v>1.0236722674665042</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <f t="shared" si="1"/>
+        <v>6.1173451588555281</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1049,8 +1245,12 @@
         <f t="shared" si="0"/>
         <v>1.0268338904464611</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <f t="shared" si="1"/>
+        <v>7.0985183030218195</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1064,8 +1264,12 @@
         <f t="shared" si="0"/>
         <v>1.019882466084824</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42">
+        <f t="shared" si="1"/>
+        <v>5.4007553988290056</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1079,8 +1283,12 @@
         <f t="shared" si="0"/>
         <v>1.0190316641856296</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43">
+        <f t="shared" si="1"/>
+        <v>5.2724339701044869</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1094,8 +1302,12 @@
         <f t="shared" si="0"/>
         <v>1.0219500777464912</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44">
+        <f t="shared" si="1"/>
+        <v>6.1966665284318765</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1109,8 +1321,12 @@
         <f t="shared" si="0"/>
         <v>1.0211164634824721</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45">
+        <f t="shared" si="1"/>
+        <v>6.0921828436501073</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1124,8 +1340,12 @@
         <f t="shared" si="0"/>
         <v>1.0201705711483944</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46">
+        <f t="shared" si="1"/>
+        <v>5.9421719890813165</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1139,8 +1359,12 @@
         <f t="shared" si="0"/>
         <v>1.019870778717693</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47">
+        <f t="shared" si="1"/>
+        <v>5.9719298870288071</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1154,8 +1378,12 @@
         <f t="shared" si="0"/>
         <v>1.0213773200734859</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <f t="shared" si="1"/>
+        <v>6.5523671088576521</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1169,8 +1397,12 @@
         <f t="shared" si="0"/>
         <v>1.021804407050354</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <f t="shared" si="1"/>
+        <v>6.8261441122833162</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1185,7 +1417,7 @@
         <v>1.10379641997152</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1195,15 +1427,14 @@
       <c r="C51">
         <v>353.09203786649988</v>
       </c>
-      <c r="E51">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E54" s="3">
-        <f>SUM(E2:E50)/49</f>
-        <v>1.0785879596190182</v>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E54" s="3"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F55" s="4">
+        <f>SUM(F2:F49)/48</f>
+        <v>6.4523707757581166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>